<commit_message>
Order list: U1 back to BQ7695203PFBR (proven on the working board)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U1Rdq73FHAWn7HLCu1GGMU
</commit_message>
<xml_diff>
--- a/Hardware/BMS_V4/BOM/BMS_V4.02_Order_List.xlsx
+++ b/Hardware/BMS_V4/BOM/BMS_V4.02_Order_List.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="297">
   <si>
     <t xml:space="preserve">BMS v4.02 - purchase list</t>
   </si>
@@ -812,16 +812,16 @@
     <t xml:space="preserve">Ekom</t>
   </si>
   <si>
-    <t xml:space="preserve">BQ7695201PFBR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Battery monitor 3-16S, SPI + CRC, REG1 off, TQFP-48</t>
+    <t xml:space="preserve">BQ7695203PFBR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battery monitor 3-16S, SPI + CRC, TQFP-48</t>
   </si>
   <si>
     <t xml:space="preserve">U1</t>
   </si>
   <si>
-    <t xml:space="preserve">NOT BQ7695203: its MISO is driven from REG1, which has no supply on this board (REGIN = GND), so SPI would not work. Price/stock to find</t>
+    <t xml:space="preserve">Same variant as on the working v4.013 board (proven with this firmware)</t>
   </si>
   <si>
     <t xml:space="preserve">CD74HC4067SM96</t>
@@ -4620,42 +4620,46 @@
       <c r="N74" s="7"/>
     </row>
     <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="10" t="n">
+      <c r="A75" s="6" t="n">
         <v>70</v>
       </c>
-      <c r="B75" s="10" t="s">
+      <c r="B75" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="C75" s="10" t="s">
+      <c r="C75" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="D75" s="10" t="s">
+      <c r="D75" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="E75" s="11" t="s">
+      <c r="E75" s="7" t="s">
         <v>263</v>
       </c>
-      <c r="F75" s="11" t="s">
+      <c r="F75" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="G75" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H75" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I75" s="10" t="n">
+      <c r="G75" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H75" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I75" s="6" t="n">
         <f aca="false">MAX(H75,CEILING(G75*$D$3,H75))</f>
         <v>2</v>
       </c>
-      <c r="J75" s="12"/>
-      <c r="K75" s="12" t="str">
+      <c r="J75" s="8" t="n">
+        <v>421.52</v>
+      </c>
+      <c r="K75" s="8" t="n">
         <f aca="false">IF(J75="","",J75*I75)</f>
-        <v/>
-      </c>
-      <c r="L75" s="10"/>
-      <c r="M75" s="10"/>
-      <c r="N75" s="11" t="s">
+        <v>843.04</v>
+      </c>
+      <c r="L75" s="6"/>
+      <c r="M75" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="N75" s="7" t="s">
         <v>265</v>
       </c>
     </row>
@@ -4732,7 +4736,7 @@
       </c>
       <c r="K78" s="17" t="n">
         <f aca="false">SUM(K6:K76)</f>
-        <v>3397.97397</v>
+        <v>4241.01397</v>
       </c>
       <c r="L78" s="14"/>
       <c r="M78" s="14"/>
@@ -4774,7 +4778,7 @@
       </c>
       <c r="K80" s="16" t="n">
         <f aca="false">SUMIF(B6:B76,"Ekom",K6:K76)</f>
-        <v>0</v>
+        <v>843.04</v>
       </c>
       <c r="L80" s="14"/>
       <c r="M80" s="14"/>
@@ -4870,7 +4874,8 @@
     <hyperlink ref="M72" r:id="rId67" display="open"/>
     <hyperlink ref="M73" r:id="rId68" display="open"/>
     <hyperlink ref="M74" r:id="rId69" display="open"/>
-    <hyperlink ref="M76" r:id="rId70" display="open"/>
+    <hyperlink ref="M75" r:id="rId70" display="open"/>
+    <hyperlink ref="M76" r:id="rId71" display="open"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4879,7 +4884,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId71"/>
+  <drawing r:id="rId72"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Order list: U1 = BQ7695204PFBR (SPI+CRC, REG1 3.3 V default)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U1Rdq73FHAWn7HLCu1GGMU
</commit_message>
<xml_diff>
--- a/Hardware/BMS_V4/BOM/BMS_V4.02_Order_List.xlsx
+++ b/Hardware/BMS_V4/BOM/BMS_V4.02_Order_List.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="297">
   <si>
     <t xml:space="preserve">BMS v4.02 - purchase list</t>
   </si>
@@ -812,16 +812,16 @@
     <t xml:space="preserve">Ekom</t>
   </si>
   <si>
-    <t xml:space="preserve">BQ7695203PFBR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Battery monitor 3-16S, SPI + CRC, TQFP-48</t>
+    <t xml:space="preserve">BQ7695204PFBR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Battery monitor 3-16S, SPI + CRC, REG1 3.3V default, TQFP-48</t>
   </si>
   <si>
     <t xml:space="preserve">U1</t>
   </si>
   <si>
-    <t xml:space="preserve">Same variant as on the working v4.013 board (proven with this firmware)</t>
+    <t xml:space="preserve">Price and supplier to find. Works on v4.02 like the BQ7695203 (REG1 unpowered); also safe for v4.03 (REG1 starts at 3.3 V). Fallback: BQ7695203PFBR at Ekom, 421.52 TRY</t>
   </si>
   <si>
     <t xml:space="preserve">CD74HC4067SM96</t>
@@ -4619,47 +4619,43 @@
       </c>
       <c r="N74" s="7"/>
     </row>
-    <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="6" t="n">
+    <row r="75" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="B75" s="6" t="s">
+      <c r="B75" s="10" t="s">
         <v>261</v>
       </c>
-      <c r="C75" s="6" t="s">
+      <c r="C75" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D75" s="6" t="s">
+      <c r="D75" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="E75" s="7" t="s">
+      <c r="E75" s="11" t="s">
         <v>263</v>
       </c>
-      <c r="F75" s="7" t="s">
+      <c r="F75" s="11" t="s">
         <v>264</v>
       </c>
-      <c r="G75" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H75" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I75" s="6" t="n">
+      <c r="G75" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H75" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I75" s="10" t="n">
         <f aca="false">MAX(H75,CEILING(G75*$D$3,H75))</f>
         <v>2</v>
       </c>
-      <c r="J75" s="8" t="n">
-        <v>421.52</v>
-      </c>
-      <c r="K75" s="8" t="n">
+      <c r="J75" s="12"/>
+      <c r="K75" s="12" t="str">
         <f aca="false">IF(J75="","",J75*I75)</f>
-        <v>843.04</v>
-      </c>
-      <c r="L75" s="6"/>
-      <c r="M75" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="N75" s="7" t="s">
+        <v/>
+      </c>
+      <c r="L75" s="10"/>
+      <c r="M75" s="10"/>
+      <c r="N75" s="11" t="s">
         <v>265</v>
       </c>
     </row>
@@ -4736,7 +4732,7 @@
       </c>
       <c r="K78" s="17" t="n">
         <f aca="false">SUM(K6:K76)</f>
-        <v>4241.01397</v>
+        <v>3397.97397</v>
       </c>
       <c r="L78" s="14"/>
       <c r="M78" s="14"/>
@@ -4778,7 +4774,7 @@
       </c>
       <c r="K80" s="16" t="n">
         <f aca="false">SUMIF(B6:B76,"Ekom",K6:K76)</f>
-        <v>843.04</v>
+        <v>0</v>
       </c>
       <c r="L80" s="14"/>
       <c r="M80" s="14"/>
@@ -4874,8 +4870,7 @@
     <hyperlink ref="M72" r:id="rId67" display="open"/>
     <hyperlink ref="M73" r:id="rId68" display="open"/>
     <hyperlink ref="M74" r:id="rId69" display="open"/>
-    <hyperlink ref="M75" r:id="rId70" display="open"/>
-    <hyperlink ref="M76" r:id="rId71" display="open"/>
+    <hyperlink ref="M76" r:id="rId70" display="open"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4884,7 +4879,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId72"/>
+  <drawing r:id="rId71"/>
 </worksheet>
 </file>
 

</xml_diff>